<commit_message>
feat: refined prompt responses for clarity in the "prompt_CBs_and_CB_Pairs.json" JSON file + updated "CBs_and_CB_Pairs.xlsx" Excel files (in the "data\describe\" & "\data\gpt_examples\" folders/directories).
</commit_message>
<xml_diff>
--- a/data/describe/CBs_and_CB_Pairs.xlsx
+++ b/data/describe/CBs_and_CB_Pairs.xlsx
@@ -901,12 +901,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CBs or CB-Pairs holding metrics with z-score values: 
-- `≥ 1.5` = Outstanding, 
-- `1.5 &gt; z ≥ 1.0` = Excellent, 
-- `1.0 &gt; z ≥ 0.5` = Good, 
-- `0.5 &gt; z ≥ -0.5` = Average, 
-- `-0.5 &gt; z ≥ -1.0` = Below Average, 
+          <t>The interpretation mappings being used for different z-score ranges or values of (quality-related, fit-related, and component-related) metrics for the individual CBs, CB-Pairs, and Anchor CB-Companion CB analysis task type settings are:
+- `z ≥ 1.5` = Outstanding,
+- `1.5 &gt; z ≥ 1.0` = Excellent,
+- `1.0 &gt; z ≥ 0.5` = Good,
+- `0.5 &gt; z ≥ -0.5` = Average,
+- `-0.5 &gt; z ≥ -1.0` = Below Average, and
 - `-1.0 &gt; z` = Poor.</t>
         </is>
       </c>
@@ -2010,8 +2010,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Happy to — there's always room for one more well-drilled CB duo in the back line... who would you like to know about next? 
-Please select them from the drop-down list on the left!</t>
+          <t>Happy to — there's always room for one more well-drilled CB duo in the back line... who would you like to know about next?</t>
         </is>
       </c>
     </row>

</xml_diff>